<commit_message>
Actualizacao da pagina da Beira
</commit_message>
<xml_diff>
--- a/Pegada_Baseline_2026.xlsx
+++ b/Pegada_Baseline_2026.xlsx
@@ -1363,11 +1363,11 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46199.0</v>
+        <v>46196.0</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Anabela Fernardo</t>
+          <t>Karina Sissa Machava</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>5.	Carvão,6.	Lenha,9.	Não utiliza energia</t>
+          <t>9.	Não utiliza energia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Nunca</t>
+          <t>Não se aplica</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Compra dentro do meu bairro.</t>
+          <t>Dentro da cidade (mas fora do bairro)</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Compra sempre que precisa.</t>
+          <t>Compra a grosso 3-4 vezes na semana/mês (a depender do negocio)</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>O meu negócio não utiliza embalagens</t>
+          <t>Embalagens de plástico</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1457,17 +1457,17 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Sempre adquire produtos vendidos em embalagens plásticas.</t>
+          <t>As vezes adquire produtos vendidos em embalagens plásticas.</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t/>
+          <t>As vezes utiliza meios de deslocação que tem baixa emissão de gases</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -1487,12 +1487,12 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Nunca reutiliza o lixo não orgânico dentro do negócio.</t>
+          <t>As vezes reutiliza o lixo não orgânico dentro do negócio.</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Nunca reutiliza agua para desempenhar atividades do negocio.</t>
+          <t>As vezes reutiliza agua para desempenhar atividades do negocio.</t>
         </is>
       </c>
     </row>
@@ -1503,11 +1503,11 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46196.0</v>
+        <v>46224.0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Karina Sissa Machava</t>
+          <t>Anabela Fernardo</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1542,12 +1542,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Ângela Antonio Manuel Bene</t>
+          <t>Anita Sábado Araújo</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9.	Não utiliza energia</t>
+          <t>5.	Carvão,6.	Lenha,9.	Não utiliza energia</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Nunca</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Dentro da cidade (mas fora do bairro)</t>
+          <t>Compra dentro do meu bairro.</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Compra a grosso 3-4 vezes na semana/mês (a depender do negocio)</t>
+          <t>Compra sempre que precisa.</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Embalagens de plástico</t>
+          <t>O meu negócio não utiliza embalagens</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>As vezes adquire produtos vendidos em embalagens plásticas.</t>
+          <t>Sempre adquire produtos vendidos em embalagens plásticas.</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>As vezes utiliza meios de deslocação que tem baixa emissão de gases</t>
+          <t/>
         </is>
       </c>
       <c r="X11" t="inlineStr">
@@ -1627,12 +1627,12 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>As vezes reutiliza o lixo não orgânico dentro do negócio.</t>
+          <t>Nunca reutiliza o lixo não orgânico dentro do negócio.</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>As vezes reutiliza agua para desempenhar atividades do negocio.</t>
+          <t>Nunca reutiliza agua para desempenhar atividades do negocio.</t>
         </is>
       </c>
     </row>
@@ -12388,22 +12388,22 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{482C6D38-3E48-461B-939A-6164662AA0F5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B17A6A24-FBEC-4203-8431-D3383679F2BF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A571D4AC-D58A-46B3-BE3B-34C29FF6DC99}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3394BA16-AC50-4299-AE7F-40ED9534DC63}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5E3D361-17AB-4C2F-8795-C0843FEA74C7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86B5F24E-09F7-4D8B-B1B8-BB2188FBEEF6}"/>
 </file>
</xml_diff>